<commit_message>
hiring-sheet: keep only direct LinkedIn JD links (25 verified roles)
</commit_message>
<xml_diff>
--- a/linkedin-content-plan/answers/hiring-sheet.xlsx
+++ b/linkedin-content-plan/answers/hiring-sheet.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hiring Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hiring Sheet'!$A$1:$G$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hiring Sheet'!$A$1:$G$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1388,253 +1388,8 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Walmart Global Tech</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>Open Walmart careers (DE filter)</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>Bengaluru / Chennai</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>https://careers.walmart.com/results?q=data%20engineer&amp;page=1&amp;sort=rank</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>Swiggy</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>Open Swiggy careers</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>Bengaluru, India</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>https://careers.swiggy.com/</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>Tiger Analytics</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Consulting</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>Open Tiger careers</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>Chennai / Bengaluru / Remote</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>https://careers.tigeranalytics.com/jobs/</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>LatentView Analytics</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Consulting</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>Open LatentView careers</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>Chennai, India</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>https://latentview.com/careers/</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>PhonePe</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>Open PhonePe careers</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>Bengaluru, India</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>https://www.phonepe.com/careers/job-openings/</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>CRED</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>Open CRED careers</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>Bengaluru, India</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>https://careers.cred.club/</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>Zerodha</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>Open Zerodha careers</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>Bengaluru, India</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>https://zerodha.com/careers/</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G33"/>
+  <autoFilter ref="A1:G26"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -1661,13 +1416,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
hiring-sheet: 47 roles (25 direct JDs + 22 live LinkedIn searches)
</commit_message>
<xml_diff>
--- a/linkedin-content-plan/answers/hiring-sheet.xlsx
+++ b/linkedin-content-plan/answers/hiring-sheet.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hiring Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hiring Sheet'!$A$1:$G$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hiring Sheet'!$A$1:$G$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -473,7 +473,7 @@
     <col width="38" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1388,8 +1388,778 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Walmart Global Tech</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Senior Data Engineer</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20Walmart%20Global%20Tech&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Walmart Global Tech</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Staff Data Engineer</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Staff%20Data%20Engineer%20Walmart%20Global%20Tech&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Walmart Global Tech</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Data Engineer III - Streaming</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Data%20Engineer%20III%20-%20Streaming%20Walmart%20Global%20Tech&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Walmart Global Tech</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Data Engineer - Analytics</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Chennai, India</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Data%20Engineer%20-%20Analytics%20Walmart%20Global%20Tech&amp;location=Chennai%2C%20Tamil%20Nadu%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Swiggy</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Data Engineer II</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Data%20Engineer%20II%20Swiggy&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Swiggy</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Senior Data Engineer</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20Swiggy&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Swiggy</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Data Engineer - Realtime</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Data%20Engineer%20-%20Realtime%20Swiggy&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Swiggy</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Lead Data Engineer</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Lead%20Data%20Engineer%20Swiggy&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>PhonePe</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Data%20Engineer%20PhonePe&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>PhonePe</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Senior Data Engineer</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20PhonePe&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>PhonePe</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Data Platform Engineer</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Data%20Platform%20Engineer%20PhonePe&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Tiger Analytics</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Consulting</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Chennai, India</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Data%20Engineer%20Tiger%20Analytics&amp;location=Chennai%2C%20Tamil%20Nadu%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Tiger Analytics</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Consulting</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Senior Data Engineer</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20Tiger%20Analytics&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Tiger Analytics</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Consulting</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Azure Data Engineer</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>India (Remote)</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Azure%20Data%20Engineer%20Tiger%20Analytics&amp;location=India</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>LatentView Analytics</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Consulting</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Chennai, India</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Data%20Engineer%20LatentView%20Analytics&amp;location=Chennai%2C%20Tamil%20Nadu%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>LatentView Analytics</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Consulting</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Senior Data Engineer</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Chennai, India</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20LatentView%20Analytics&amp;location=Chennai%2C%20Tamil%20Nadu%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>CRED</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Senior Data Engineer</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20CRED&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Zerodha</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Senior Data Engineer</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20Zerodha&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Data%20Engineer%20Groww&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Ola Krutrim</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Senior Data Engineer</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20Ola%20Krutrim&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Uber</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Senior Data Engineer</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20Uber&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Atlassian</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Senior Data Engineer</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20Atlassian&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G26"/>
+  <autoFilter ref="A1:G48"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -1416,6 +2186,28 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId47"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
hiring-sheet: add Find Recruiter (live LinkedIn search) + outreach tracker columns
</commit_message>
<xml_diff>
--- a/linkedin-content-plan/answers/hiring-sheet.xlsx
+++ b/linkedin-content-plan/answers/hiring-sheet.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hiring Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hiring Sheet'!$A$1:$G$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hiring Sheet'!$A$1:$L$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -86,7 +86,7 @@
       <protection locked="0" hidden="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -97,6 +97,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -464,19 +467,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Sr</t>
@@ -510,6 +518,31 @@
       <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Direct JD Link</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Find Recruiter</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Recruiter Name</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Recruiter LinkedIn</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Outreach Status</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Last Contact</t>
         </is>
       </c>
     </row>
@@ -547,6 +580,15 @@
           <t>https://www.linkedin.com/jobs/view/4414589448/</t>
         </is>
       </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="n"/>
+      <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -582,6 +624,15 @@
           <t>https://www.linkedin.com/jobs/view/4342937817/</t>
         </is>
       </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -617,6 +668,15 @@
           <t>https://www.linkedin.com/jobs/view/4385853976/</t>
         </is>
       </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -652,6 +712,15 @@
           <t>https://www.linkedin.com/jobs/view/4384166827/</t>
         </is>
       </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -687,6 +756,15 @@
           <t>https://www.linkedin.com/jobs/view/4402986402/</t>
         </is>
       </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -722,6 +800,15 @@
           <t>https://www.linkedin.com/jobs/view/4405342001/</t>
         </is>
       </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -757,6 +844,15 @@
           <t>https://www.linkedin.com/jobs/view/4405980075/</t>
         </is>
       </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="n"/>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -792,6 +888,15 @@
           <t>https://www.linkedin.com/jobs/view/4414469550/</t>
         </is>
       </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="n"/>
+      <c r="K9" s="3" t="n"/>
+      <c r="L9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -827,6 +932,15 @@
           <t>https://www.linkedin.com/jobs/view/4407345092/</t>
         </is>
       </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="n"/>
+      <c r="K10" s="3" t="n"/>
+      <c r="L10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -862,6 +976,15 @@
           <t>https://www.linkedin.com/jobs/view/4409767662/</t>
         </is>
       </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="n"/>
+      <c r="J11" s="3" t="n"/>
+      <c r="K11" s="3" t="n"/>
+      <c r="L11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -897,6 +1020,15 @@
           <t>https://www.linkedin.com/jobs/view/4412882944/</t>
         </is>
       </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="n"/>
+      <c r="J12" s="3" t="n"/>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -932,6 +1064,15 @@
           <t>https://www.linkedin.com/jobs/view/4412245982/</t>
         </is>
       </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="n"/>
+      <c r="J13" s="3" t="n"/>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -967,6 +1108,15 @@
           <t>https://www.linkedin.com/jobs/view/4407279012/</t>
         </is>
       </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="n"/>
+      <c r="J14" s="3" t="n"/>
+      <c r="K14" s="3" t="n"/>
+      <c r="L14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
@@ -1002,6 +1152,15 @@
           <t>https://www.linkedin.com/jobs/view/4372694125/</t>
         </is>
       </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="n"/>
+      <c r="J15" s="3" t="n"/>
+      <c r="K15" s="3" t="n"/>
+      <c r="L15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -1037,6 +1196,15 @@
           <t>https://www.linkedin.com/jobs/view/4407819630/</t>
         </is>
       </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="n"/>
+      <c r="J16" s="3" t="n"/>
+      <c r="K16" s="3" t="n"/>
+      <c r="L16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -1072,6 +1240,15 @@
           <t>https://www.linkedin.com/jobs/view/4410026155/</t>
         </is>
       </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="n"/>
+      <c r="J17" s="3" t="n"/>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -1107,6 +1284,15 @@
           <t>https://www.linkedin.com/jobs/view/4409894934/</t>
         </is>
       </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="n"/>
+      <c r="J18" s="3" t="n"/>
+      <c r="K18" s="3" t="n"/>
+      <c r="L18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
@@ -1142,6 +1328,15 @@
           <t>https://www.linkedin.com/jobs/view/4407824357/</t>
         </is>
       </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="n"/>
+      <c r="J19" s="3" t="n"/>
+      <c r="K19" s="3" t="n"/>
+      <c r="L19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -1177,6 +1372,15 @@
           <t>https://www.linkedin.com/jobs/view/4416254012/</t>
         </is>
       </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="n"/>
+      <c r="J20" s="3" t="n"/>
+      <c r="K20" s="3" t="n"/>
+      <c r="L20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -1212,6 +1416,15 @@
           <t>https://www.linkedin.com/jobs/view/4416218040/</t>
         </is>
       </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="n"/>
+      <c r="J21" s="3" t="n"/>
+      <c r="K21" s="3" t="n"/>
+      <c r="L21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -1247,6 +1460,15 @@
           <t>https://www.linkedin.com/jobs/view/4416095682/</t>
         </is>
       </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="n"/>
+      <c r="J22" s="3" t="n"/>
+      <c r="K22" s="3" t="n"/>
+      <c r="L22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -1282,6 +1504,15 @@
           <t>https://www.linkedin.com/jobs/view/4359195677/</t>
         </is>
       </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="n"/>
+      <c r="J23" s="3" t="n"/>
+      <c r="K23" s="3" t="n"/>
+      <c r="L23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -1317,6 +1548,15 @@
           <t>https://www.linkedin.com/jobs/view/4375715959/</t>
         </is>
       </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="n"/>
+      <c r="J24" s="3" t="n"/>
+      <c r="K24" s="3" t="n"/>
+      <c r="L24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -1352,6 +1592,15 @@
           <t>https://www.linkedin.com/jobs/view/4391701394/</t>
         </is>
       </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="n"/>
+      <c r="J25" s="3" t="n"/>
+      <c r="K25" s="3" t="n"/>
+      <c r="L25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -1387,6 +1636,15 @@
           <t>https://www.linkedin.com/jobs/view/4392996596/</t>
         </is>
       </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="n"/>
+      <c r="J26" s="3" t="n"/>
+      <c r="K26" s="3" t="n"/>
+      <c r="L26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
@@ -1422,6 +1680,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20Walmart%20Global%20Tech&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
         </is>
       </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="n"/>
+      <c r="J27" s="3" t="n"/>
+      <c r="K27" s="3" t="n"/>
+      <c r="L27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
@@ -1457,6 +1724,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Staff%20Data%20Engineer%20Walmart%20Global%20Tech&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
         </is>
       </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+      <c r="K28" s="3" t="n"/>
+      <c r="L28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -1492,6 +1768,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Data%20Engineer%20III%20-%20Streaming%20Walmart%20Global%20Tech&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
         </is>
       </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="n"/>
+      <c r="J29" s="3" t="n"/>
+      <c r="K29" s="3" t="n"/>
+      <c r="L29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
@@ -1527,6 +1812,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Data%20Engineer%20-%20Analytics%20Walmart%20Global%20Tech&amp;location=Chennai%2C%20Tamil%20Nadu%2C%20India</t>
         </is>
       </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="n"/>
+      <c r="J30" s="3" t="n"/>
+      <c r="K30" s="3" t="n"/>
+      <c r="L30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
@@ -1562,6 +1856,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Data%20Engineer%20II%20Swiggy&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
         </is>
       </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="n"/>
+      <c r="J31" s="3" t="n"/>
+      <c r="K31" s="3" t="n"/>
+      <c r="L31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
@@ -1597,6 +1900,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20Swiggy&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
         </is>
       </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="n"/>
+      <c r="J32" s="3" t="n"/>
+      <c r="K32" s="3" t="n"/>
+      <c r="L32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
@@ -1632,6 +1944,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Data%20Engineer%20-%20Realtime%20Swiggy&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
         </is>
       </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="n"/>
+      <c r="J33" s="3" t="n"/>
+      <c r="K33" s="3" t="n"/>
+      <c r="L33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
@@ -1667,6 +1988,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Lead%20Data%20Engineer%20Swiggy&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
         </is>
       </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="n"/>
+      <c r="J34" s="3" t="n"/>
+      <c r="K34" s="3" t="n"/>
+      <c r="L34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
@@ -1702,6 +2032,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Data%20Engineer%20PhonePe&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
         </is>
       </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="n"/>
+      <c r="J35" s="3" t="n"/>
+      <c r="K35" s="3" t="n"/>
+      <c r="L35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -1737,6 +2076,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20PhonePe&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
         </is>
       </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="n"/>
+      <c r="J36" s="3" t="n"/>
+      <c r="K36" s="3" t="n"/>
+      <c r="L36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
@@ -1772,6 +2120,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Data%20Platform%20Engineer%20PhonePe&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
         </is>
       </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="n"/>
+      <c r="J37" s="3" t="n"/>
+      <c r="K37" s="3" t="n"/>
+      <c r="L37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
@@ -1807,6 +2164,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Data%20Engineer%20Tiger%20Analytics&amp;location=Chennai%2C%20Tamil%20Nadu%2C%20India</t>
         </is>
       </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="n"/>
+      <c r="J38" s="3" t="n"/>
+      <c r="K38" s="3" t="n"/>
+      <c r="L38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
@@ -1842,6 +2208,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20Tiger%20Analytics&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
         </is>
       </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="n"/>
+      <c r="J39" s="3" t="n"/>
+      <c r="K39" s="3" t="n"/>
+      <c r="L39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
@@ -1877,6 +2252,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Azure%20Data%20Engineer%20Tiger%20Analytics&amp;location=India</t>
         </is>
       </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="n"/>
+      <c r="J40" s="3" t="n"/>
+      <c r="K40" s="3" t="n"/>
+      <c r="L40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
@@ -1912,6 +2296,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Data%20Engineer%20LatentView%20Analytics&amp;location=Chennai%2C%20Tamil%20Nadu%2C%20India</t>
         </is>
       </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="n"/>
+      <c r="J41" s="3" t="n"/>
+      <c r="K41" s="3" t="n"/>
+      <c r="L41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n">
@@ -1947,6 +2340,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20LatentView%20Analytics&amp;location=Chennai%2C%20Tamil%20Nadu%2C%20India</t>
         </is>
       </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="n"/>
+      <c r="J42" s="3" t="n"/>
+      <c r="K42" s="3" t="n"/>
+      <c r="L42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n">
@@ -1982,6 +2384,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20CRED&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
         </is>
       </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="n"/>
+      <c r="J43" s="3" t="n"/>
+      <c r="K43" s="3" t="n"/>
+      <c r="L43" s="3" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n">
@@ -2017,6 +2428,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20Zerodha&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
         </is>
       </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="n"/>
+      <c r="J44" s="3" t="n"/>
+      <c r="K44" s="3" t="n"/>
+      <c r="L44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n">
@@ -2052,6 +2472,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Data%20Engineer%20Groww&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
         </is>
       </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="n"/>
+      <c r="J45" s="3" t="n"/>
+      <c r="K45" s="3" t="n"/>
+      <c r="L45" s="3" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
@@ -2087,6 +2516,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20Ola%20Krutrim&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
         </is>
       </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="n"/>
+      <c r="J46" s="3" t="n"/>
+      <c r="K46" s="3" t="n"/>
+      <c r="L46" s="3" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n">
@@ -2122,6 +2560,15 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20Uber&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
         </is>
       </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="n"/>
+      <c r="J47" s="3" t="n"/>
+      <c r="K47" s="3" t="n"/>
+      <c r="L47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
@@ -2157,57 +2604,118 @@
           <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Data%20Engineer%20Atlassian&amp;location=Bengaluru%2C%20Karnataka%2C%20India</t>
         </is>
       </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>🔍 Find recruiter</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="n"/>
+      <c r="J48" s="3" t="n"/>
+      <c r="K48" s="3" t="n"/>
+      <c r="L48" s="3" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G48"/>
+  <autoFilter ref="A1:L48"/>
+  <dataValidations count="1">
+    <dataValidation sqref="K2:K48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Not contacted,DM sent,Reply received,Interviewed,Rejected,Offer"</formula1>
+    </dataValidation>
+  </dataValidations>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId94"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>